<commit_message>
Se extraen las etiquetas de los valores para crear las tablas de dimensiones para el informe en Power BI
</commit_message>
<xml_diff>
--- a/bitacora/renombrar_niveles.xlsx
+++ b/bitacora/renombrar_niveles.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Prog\tesis\datos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Prog\tesis\bitacora\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9036DCD6-0C3C-4D95-90E0-81DCDFCD3374}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED1652AC-D824-449F-87BD-F300A92EBC5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1068" yWindow="-108" windowWidth="22080" windowHeight="13176" activeTab="2" xr2:uid="{625366E0-2D2B-4A7F-B490-7752D575F381}"/>
   </bookViews>

</xml_diff>